<commit_message>
Fix some database-related errors
</commit_message>
<xml_diff>
--- a/Data/ConfigRuntime.xlsx
+++ b/Data/ConfigRuntime.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E_MMH242\Documents\UiPath\Template\ExtendedREFramework_Reporter\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E_MMH242\Documents\UiPath\Templates\ExtendedREFramework_Reporter\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -16,14 +16,64 @@
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
     <sheet name="Credentials" sheetId="5" r:id="rId4"/>
-    <sheet name="Paths" sheetId="7" r:id="rId5"/>
+    <sheet name="Drives" sheetId="8" r:id="rId5"/>
+    <sheet name="Paths" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>MORELL HIGUERAS, MARC</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>You can use this as the BasePathName in sheet Paths</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Name within sheet Assets containing the value of the path to map onto the drive</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Drives should only be mapped when a credential is required to access a network resource. Otherwise, use the server path.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="167">
   <si>
     <t>Name</t>
   </si>
@@ -527,12 +577,33 @@
   <si>
     <t>DispatcherJob,PerformerJob</t>
   </si>
+  <si>
+    <t>CheckReadyToReport</t>
+  </si>
+  <si>
+    <t>If enabled, runs the "CheckIsReadyToReport" workflow. By default ensures the queue has no pending items before reporting.</t>
+  </si>
+  <si>
+    <t>MinutesSuspended</t>
+  </si>
+  <si>
+    <t>When CheckReadyToReport is true, amount of minutes the job will be suspended between readiness checks. Must be an integer value.</t>
+  </si>
+  <si>
+    <t>Letter</t>
+  </si>
+  <si>
+    <t>Asset Path</t>
+  </si>
+  <si>
+    <t>Credential</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -569,6 +640,19 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -596,7 +680,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -611,6 +695,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -925,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z1023"/>
+  <dimension ref="A1:Z1024"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1008,232 +1101,235 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="4"/>
+    <row r="6" spans="1:26" ht="30">
+      <c r="A6" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B6" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="7" spans="1:26">
-      <c r="A7" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="4"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="11"/>
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="30">
-      <c r="A12" t="s">
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="30">
+      <c r="A13" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:26">
-      <c r="B13" s="2"/>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>114</v>
-      </c>
-      <c r="B14" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>115</v>
-      </c>
+    <row r="14" spans="1:26">
+      <c r="B14" s="2"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" t="s">
-        <v>56</v>
+        <v>114</v>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>51</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>106</v>
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>56</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>107</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>116</v>
-      </c>
-      <c r="B17" t="b">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B18" t="b">
         <v>0</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B19" t="b">
         <v>0</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
         <v>120</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
-        <v>148</v>
-      </c>
-      <c r="B22" t="b">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
-        <v>150</v>
-      </c>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>152</v>
-      </c>
-      <c r="B23" t="s">
-        <v>154</v>
+        <v>148</v>
+      </c>
+      <c r="B23" t="b">
+        <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>156</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>157</v>
+        <v>152</v>
+      </c>
+      <c r="B24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>147</v>
-      </c>
-      <c r="B25" t="s">
-        <v>159</v>
-      </c>
-      <c r="C25" t="s">
-        <v>149</v>
+        <v>156</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A27" t="s">
         <v>151</v>
       </c>
-      <c r="B26" t="b">
+      <c r="B27" t="b">
         <v>1</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1">
-      <c r="C27" s="4"/>
-    </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A28" s="2" t="s">
+      <c r="C28" s="4"/>
+    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A29" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B29" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-    </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A30" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>93</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
       <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B31" s="8" t="s">
         <v>93</v>
       </c>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A32" t="s">
-        <v>99</v>
+      <c r="A32" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>93</v>
@@ -1241,23 +1337,23 @@
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B33" s="8" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>101</v>
+      <c r="A34" t="s">
+        <v>100</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A35" t="s">
-        <v>102</v>
+      <c r="A35" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="B35" s="8" t="s">
         <v>93</v>
@@ -1265,61 +1361,68 @@
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A37" t="s">
         <v>144</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B37" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C37" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B37" s="8"/>
-    </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A38" t="s">
+      <c r="B38" s="8"/>
+    </row>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
         <v>94</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="40" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A40" t="s">
-        <v>95</v>
-      </c>
-      <c r="B40" t="s">
-        <v>96</v>
-      </c>
-    </row>
+    <row r="40" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="41" spans="1:3" ht="14.25" customHeight="1">
       <c r="A41" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A42" t="s">
         <v>104</v>
       </c>
-      <c r="B41" t="b">
+      <c r="B42" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="43" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A43" t="s">
-        <v>131</v>
-      </c>
-      <c r="B43" t="s">
-        <v>129</v>
-      </c>
-    </row>
+    <row r="43" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
         <v>132</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="48" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2298,6 +2401,7 @@
     <row r="1021" ht="14.25" customHeight="1"/>
     <row r="1022" ht="14.25" customHeight="1"/>
     <row r="1023" ht="14.25" customHeight="1"/>
+    <row r="1024" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2307,7 +2411,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z949"/>
+  <dimension ref="A1:Z950"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -2372,290 +2476,300 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" s="2" t="s">
+    <row r="4" spans="1:26" ht="30">
+      <c r="A4" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="12">
+        <v>5</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" t="s">
         <v>33</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14">
-        <v>2</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
-    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
-      <c r="A17" t="s">
+    <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:3" ht="45">
+      <c r="A18" t="s">
         <v>39</v>
       </c>
-      <c r="B17" t="b">
+      <c r="B18" t="b">
         <v>1</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A20" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B20" s="7" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" t="s">
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
         <v>53</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>55</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C21" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" t="s">
-        <v>61</v>
-      </c>
-    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B27" s="2" t="b">
+      <c r="B28" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>77</v>
+        <v>47</v>
+      </c>
+      <c r="C29" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A32" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A32" s="2" t="s">
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
     </row>
-    <row r="35" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A35" s="7" t="s">
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" s="6" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A36" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
-        <v>86</v>
-      </c>
-      <c r="B36" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="C37" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1">
       <c r="A38" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
         <v>90</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="44" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="40" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
@@ -3561,6 +3675,7 @@
     <row r="947" ht="14.25" customHeight="1"/>
     <row r="948" ht="14.25" customHeight="1"/>
     <row r="949" ht="14.25" customHeight="1"/>
+    <row r="950" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5712,6 +5827,44 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="3" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18.75">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="A single uppercase letter, A-Z" sqref="B2:B27">
+      <formula1>"A,B,C,D,E,F,G,H,I,J,K,L,M,N,O,P,Q,R,S,T,U,V,W,X,Y,Z"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>

</xml_diff>